<commit_message>
feat: handle post-possession renewal rates in inventory and archive pre-possession contracts in history
</commit_message>
<xml_diff>
--- a/Tower_A_Ownership_History_Resale_v2.xlsx
+++ b/Tower_A_Ownership_History_Resale_v2.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M43"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -496,7 +496,7 @@
         <v>5500000</v>
       </c>
       <c r="M2" t="str">
-        <v>Flat A-105: Previous owner Shakuntla Gupta transferred to MADAN GOPAL SARASWAT</v>
+        <v>Flat A-105: Prior owner Shakuntla Gupta resold to MADAN GOPAL SARASWAT</v>
       </c>
     </row>
     <row r="3">
@@ -537,39 +537,39 @@
         <v>5500000</v>
       </c>
       <c r="M3" t="str">
-        <v>Flat A-203: Previous owner Sushil Kumar Burman transferred to Sarika Jain</v>
+        <v>Flat A-203: Prior owner Sushil Kumar Burman resold to Sarika Jain</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B4" t="str">
         <v>Tower A</v>
       </c>
       <c r="C4" t="str">
-        <v>Asha Mishra</v>
+        <v>Pratap Singh</v>
       </c>
       <c r="D4" t="str">
-        <v>+91 9800000205</v>
+        <v>+91 9800000204</v>
       </c>
       <c r="E4" t="str">
-        <v>18/01/2014</v>
+        <v>29/08/2014</v>
       </c>
       <c r="F4" t="str">
-        <v>06/05/2025</v>
+        <v>10/08/2024</v>
       </c>
       <c r="G4" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H4">
         <v>1600000</v>
       </c>
       <c r="I4" t="str">
-        <v>Nirmala Devi</v>
+        <v>Pratap Singh</v>
       </c>
       <c r="J4" t="str">
-        <v>+91 9800000205</v>
+        <v>+91 9800000204</v>
       </c>
       <c r="K4">
         <v>5500000</v>
@@ -578,39 +578,39 @@
         <v>5500000</v>
       </c>
       <c r="M4" t="str">
-        <v>Flat A-205: Previous owner Asha Mishra transferred to Nirmala Devi</v>
+        <v>Flat A-204: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹16,00,000) expired/renewed to Post-Possession Rate (@ ₹9,000/mo)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B5" t="str">
         <v>Tower A</v>
       </c>
       <c r="C5" t="str">
-        <v>Jyoti Dixit and Sanjay kumar Dixit</v>
+        <v>Asha Mishra</v>
       </c>
       <c r="D5" t="str">
-        <v>+91 9800000206</v>
+        <v>+91 9800000205</v>
       </c>
       <c r="E5" t="str">
-        <v>04/05/2015</v>
+        <v>18/01/2014</v>
       </c>
       <c r="F5" t="str">
-        <v>21/05/2026</v>
+        <v>06/05/2025</v>
       </c>
       <c r="G5" t="str">
         <v>resale</v>
       </c>
       <c r="H5">
-        <v>2151000</v>
+        <v>1600000</v>
       </c>
       <c r="I5" t="str">
-        <v>Sushmita Singh</v>
+        <v>Nirmala Devi</v>
       </c>
       <c r="J5" t="str">
-        <v>+91 9800000206</v>
+        <v>+91 9800000205</v>
       </c>
       <c r="K5">
         <v>5500000</v>
@@ -619,39 +619,39 @@
         <v>5500000</v>
       </c>
       <c r="M5" t="str">
-        <v>Flat A-206: Previous owner Jyoti Dixit and Sanjay kumar Dixit transferred to Sushmita Singh</v>
+        <v>Flat A-205: Prior owner Asha Mishra resold to Nirmala Devi</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>314</v>
+        <v>206</v>
       </c>
       <c r="B6" t="str">
         <v>Tower A</v>
       </c>
       <c r="C6" t="str">
-        <v>Neeru Arora</v>
+        <v>Jyoti Dixit and Sanjay kumar Dixit</v>
       </c>
       <c r="D6" t="str">
-        <v>+91 9800000314</v>
+        <v>+91 9800000206</v>
       </c>
       <c r="E6" t="str">
-        <v>07/07/2014</v>
+        <v>04/05/2015</v>
       </c>
       <c r="F6" t="str">
-        <v>01/11/2025</v>
+        <v>21/05/2026</v>
       </c>
       <c r="G6" t="str">
         <v>resale</v>
       </c>
       <c r="H6">
-        <v>1224000</v>
+        <v>2151000</v>
       </c>
       <c r="I6" t="str">
-        <v>Gaurav Gupta</v>
+        <v>Sushmita Singh</v>
       </c>
       <c r="J6" t="str">
-        <v>+91 9800000314</v>
+        <v>+91 9800000206</v>
       </c>
       <c r="K6">
         <v>5500000</v>
@@ -660,39 +660,39 @@
         <v>5500000</v>
       </c>
       <c r="M6" t="str">
-        <v>Flat A-314: Previous owner Neeru Arora transferred to Gaurav Gupta</v>
+        <v>Flat A-206: Prior owner Jyoti Dixit and Sanjay kumar Dixit resold to Sushmita Singh</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>404</v>
+        <v>212</v>
       </c>
       <c r="B7" t="str">
         <v>Tower A</v>
       </c>
       <c r="C7" t="str">
-        <v>Suman Rani</v>
+        <v>Aman Sharma</v>
       </c>
       <c r="D7" t="str">
-        <v>+91 9800000404</v>
+        <v>+91 9800000212</v>
       </c>
       <c r="E7" t="str">
-        <v>09/09/2014</v>
+        <v>11/11/2014</v>
       </c>
       <c r="F7" t="str">
-        <v>25/10/2025</v>
+        <v>10/01/2026</v>
       </c>
       <c r="G7" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H7">
-        <v>1688500</v>
+        <v>1738600</v>
       </c>
       <c r="I7" t="str">
-        <v>Vishnu Kumar Agarwal</v>
+        <v>Aman Sharma</v>
       </c>
       <c r="J7" t="str">
-        <v>+91 9800000404</v>
+        <v>+91 9800000212</v>
       </c>
       <c r="K7">
         <v>5500000</v>
@@ -701,39 +701,39 @@
         <v>5500000</v>
       </c>
       <c r="M7" t="str">
-        <v>Flat A-404: Previous owner Suman Rani transferred to Vishnu Kumar Agarwal</v>
+        <v>Flat A-212: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹17,38,600) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>410</v>
+        <v>305</v>
       </c>
       <c r="B8" t="str">
         <v>Tower A</v>
       </c>
       <c r="C8" t="str">
-        <v>Manju Arora</v>
+        <v>Kajla Dixit</v>
       </c>
       <c r="D8" t="str">
-        <v>+91 9800000410</v>
+        <v>+91 9800000305</v>
       </c>
       <c r="E8" t="str">
-        <v>05/08/2014</v>
+        <v>20/11/2014</v>
       </c>
       <c r="F8" t="str">
-        <v>01/08/2025</v>
+        <v>10/05/2025</v>
       </c>
       <c r="G8" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H8">
-        <v>1714000</v>
+        <v>1456000</v>
       </c>
       <c r="I8" t="str">
-        <v>Mamta Singh</v>
+        <v>Kajla Dixit</v>
       </c>
       <c r="J8" t="str">
-        <v>+91 9800000410</v>
+        <v>+91 9800000305</v>
       </c>
       <c r="K8">
         <v>5500000</v>
@@ -742,39 +742,39 @@
         <v>5500000</v>
       </c>
       <c r="M8" t="str">
-        <v>Flat A-410: Previous owner Manju Arora transferred to Mamta Singh</v>
+        <v>Flat A-305: Pre-Possession Contract (91mo @ ₹16000/mo, Total: ₹14,56,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>411</v>
+        <v>312</v>
       </c>
       <c r="B9" t="str">
         <v>Tower A</v>
       </c>
       <c r="C9" t="str">
-        <v>Sushma Jain</v>
+        <v>Namita Jain</v>
       </c>
       <c r="D9" t="str">
-        <v>+91 9800000411</v>
+        <v>+91 9800000312</v>
       </c>
       <c r="E9" t="str">
-        <v>01/09/2014</v>
+        <v>30/10/2014</v>
       </c>
       <c r="F9" t="str">
-        <v>13/10/2025</v>
+        <v>10/05/2025</v>
       </c>
       <c r="G9" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H9">
-        <v>1890000</v>
+        <v>1732000</v>
       </c>
       <c r="I9" t="str">
-        <v>SWATI</v>
+        <v>Namita Jain</v>
       </c>
       <c r="J9" t="str">
-        <v>+91 9800000411</v>
+        <v>+91 9800000312</v>
       </c>
       <c r="K9">
         <v>5500000</v>
@@ -783,39 +783,39 @@
         <v>5500000</v>
       </c>
       <c r="M9" t="str">
-        <v>Flat A-411: Previous owner Sushma Jain transferred to SWATI</v>
+        <v>Flat A-312: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹17,32,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>501</v>
+        <v>314</v>
       </c>
       <c r="B10" t="str">
         <v>Tower A</v>
       </c>
       <c r="C10" t="str">
-        <v>Santokh Singh</v>
+        <v>Neeru Arora</v>
       </c>
       <c r="D10" t="str">
-        <v>+91 9800000501</v>
+        <v>+91 9800000314</v>
       </c>
       <c r="E10" t="str">
-        <v>21/05/2014</v>
+        <v>07/07/2014</v>
       </c>
       <c r="F10" t="str">
-        <v>05/12/2025</v>
+        <v>01/11/2025</v>
       </c>
       <c r="G10" t="str">
         <v>resale</v>
       </c>
       <c r="H10">
-        <v>1600000</v>
+        <v>1224000</v>
       </c>
       <c r="I10" t="str">
-        <v>Sunita Gupta</v>
+        <v>Gaurav Gupta</v>
       </c>
       <c r="J10" t="str">
-        <v>+91 9800000501</v>
+        <v>+91 9800000314</v>
       </c>
       <c r="K10">
         <v>5500000</v>
@@ -824,39 +824,39 @@
         <v>5500000</v>
       </c>
       <c r="M10" t="str">
-        <v>Flat A-501: Previous owner Santokh Singh transferred to Sunita Gupta</v>
+        <v>Flat A-314: Prior owner Neeru Arora resold to Gaurav Gupta</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>502</v>
+        <v>402</v>
       </c>
       <c r="B11" t="str">
         <v>Tower A</v>
       </c>
       <c r="C11" t="str">
-        <v>Amit Agarwal</v>
+        <v>Nisha Chaturvedi</v>
       </c>
       <c r="D11" t="str">
-        <v>+91 9800000502</v>
+        <v>+91 9800000402</v>
       </c>
       <c r="E11" t="str">
-        <v>09/10/2014</v>
+        <v>28/04/2015</v>
       </c>
       <c r="F11" t="str">
-        <v>23/04/2025</v>
+        <v>10/05/2025</v>
       </c>
       <c r="G11" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H11">
-        <v>1710000</v>
+        <v>2200000</v>
       </c>
       <c r="I11" t="str">
-        <v>Jitender</v>
+        <v>Nisha Chaturvedi</v>
       </c>
       <c r="J11" t="str">
-        <v>+91 9800000502</v>
+        <v>+91 9800000402</v>
       </c>
       <c r="K11">
         <v>5500000</v>
@@ -865,39 +865,39 @@
         <v>5500000</v>
       </c>
       <c r="M11" t="str">
-        <v>Flat A-502: Previous owner Amit Agarwal transferred to Jitender</v>
+        <v>Flat A-402: Pre-Possession Contract (100mo @ ₹22000/mo, Total: ₹22,00,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>503</v>
+        <v>403</v>
       </c>
       <c r="B12" t="str">
         <v>Tower A</v>
       </c>
       <c r="C12" t="str">
-        <v>Shefali Rani Mukherji</v>
+        <v>Anita Gupta</v>
       </c>
       <c r="D12" t="str">
-        <v>+91 9800000503</v>
+        <v>+91 9800000403</v>
       </c>
       <c r="E12" t="str">
-        <v>13/03/2014</v>
+        <v>14/03/2014</v>
       </c>
       <c r="F12" t="str">
-        <v>21/01/2026</v>
+        <v>10/02/2024</v>
       </c>
       <c r="G12" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H12">
         <v>1600000</v>
       </c>
       <c r="I12" t="str">
-        <v>Manju Goyal</v>
+        <v>Anita Gupta</v>
       </c>
       <c r="J12" t="str">
-        <v>+91 9800000503</v>
+        <v>+91 9800000403</v>
       </c>
       <c r="K12">
         <v>5500000</v>
@@ -906,39 +906,39 @@
         <v>5500000</v>
       </c>
       <c r="M12" t="str">
-        <v>Flat A-503: Previous owner Shefali Rani Mukherji transferred to Manju Goyal</v>
+        <v>Flat A-403: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹16,00,000) expired/renewed to Post-Possession Rate (@ ₹12,000/mo)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>508</v>
+        <v>404</v>
       </c>
       <c r="B13" t="str">
         <v>Tower A</v>
       </c>
       <c r="C13" t="str">
-        <v>Sanjay Madan and Sandhya Madan</v>
+        <v>Suman Rani</v>
       </c>
       <c r="D13" t="str">
-        <v>+91 9800000508</v>
+        <v>+91 9800000404</v>
       </c>
       <c r="E13" t="str">
-        <v>29/04/2014</v>
+        <v>09/09/2014</v>
       </c>
       <c r="F13" t="str">
-        <v>09/04/2025</v>
+        <v>25/10/2025</v>
       </c>
       <c r="G13" t="str">
         <v>resale</v>
       </c>
       <c r="H13">
-        <v>1600000</v>
+        <v>1688500</v>
       </c>
       <c r="I13" t="str">
         <v>Vishnu Kumar Agarwal</v>
       </c>
       <c r="J13" t="str">
-        <v>+91 9800000508</v>
+        <v>+91 9800000404</v>
       </c>
       <c r="K13">
         <v>5500000</v>
@@ -947,39 +947,39 @@
         <v>5500000</v>
       </c>
       <c r="M13" t="str">
-        <v>Flat A-508: Previous owner Sanjay Madan and Sandhya Madan transferred to Vishnu Kumar Agarwal</v>
+        <v>Flat A-404: Prior owner Suman Rani resold to Vishnu Kumar Agarwal</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>603</v>
+        <v>410</v>
       </c>
       <c r="B14" t="str">
         <v>Tower A</v>
       </c>
       <c r="C14" t="str">
-        <v>Akshay Khullar</v>
+        <v>Manju Arora</v>
       </c>
       <c r="D14" t="str">
-        <v>+91 9800000603</v>
+        <v>+91 9800000410</v>
       </c>
       <c r="E14" t="str">
-        <v>13/03/2014</v>
+        <v>05/08/2014</v>
       </c>
       <c r="F14" t="str">
-        <v>09/04/2025</v>
+        <v>01/08/2025</v>
       </c>
       <c r="G14" t="str">
         <v>resale</v>
       </c>
       <c r="H14">
-        <v>1600000</v>
+        <v>1714000</v>
       </c>
       <c r="I14" t="str">
-        <v>Pooja Chand Dwivedi</v>
+        <v>Mamta Singh</v>
       </c>
       <c r="J14" t="str">
-        <v>+91 9800000603</v>
+        <v>+91 9800000410</v>
       </c>
       <c r="K14">
         <v>5500000</v>
@@ -988,39 +988,39 @@
         <v>5500000</v>
       </c>
       <c r="M14" t="str">
-        <v>Flat A-603: Previous owner Akshay Khullar transferred to Pooja Chand Dwivedi</v>
+        <v>Flat A-410: Prior owner Manju Arora resold to Mamta Singh</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>606</v>
+        <v>411</v>
       </c>
       <c r="B15" t="str">
         <v>Tower A</v>
       </c>
       <c r="C15" t="str">
-        <v>Rajeev Varshney</v>
+        <v>Sushma Jain</v>
       </c>
       <c r="D15" t="str">
-        <v>+91 9800000606</v>
+        <v>+91 9800000411</v>
       </c>
       <c r="E15" t="str">
-        <v>10/10/2014</v>
+        <v>01/09/2014</v>
       </c>
       <c r="F15" t="str">
-        <v>21/11/2025</v>
+        <v>13/10/2025</v>
       </c>
       <c r="G15" t="str">
         <v>resale</v>
       </c>
       <c r="H15">
-        <v>1591800</v>
+        <v>1890000</v>
       </c>
       <c r="I15" t="str">
-        <v>Praveen Tripathi</v>
+        <v>SWATI</v>
       </c>
       <c r="J15" t="str">
-        <v>+91 9800000606</v>
+        <v>+91 9800000411</v>
       </c>
       <c r="K15">
         <v>5500000</v>
@@ -1029,39 +1029,39 @@
         <v>5500000</v>
       </c>
       <c r="M15" t="str">
-        <v>Flat A-606: Previous owner Rajeev Varshney transferred to Praveen Tripathi</v>
+        <v>Flat A-411: Prior owner Sushma Jain resold to SWATI</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>610</v>
+        <v>413</v>
       </c>
       <c r="B16" t="str">
         <v>Tower A</v>
       </c>
       <c r="C16" t="str">
-        <v>Jitender Kumar</v>
+        <v>Geeta Giri</v>
       </c>
       <c r="D16" t="str">
-        <v>+91 9800000610</v>
+        <v>+91 9800000413</v>
       </c>
       <c r="E16" t="str">
-        <v>21/10/2014</v>
+        <v>07/07/2014</v>
       </c>
       <c r="F16" t="str">
-        <v>13/03/2026</v>
+        <v>10/07/2024</v>
       </c>
       <c r="G16" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H16">
-        <v>1875000</v>
+        <v>1716000</v>
       </c>
       <c r="I16" t="str">
-        <v>Sudheer Rai</v>
+        <v>Geeta Giri</v>
       </c>
       <c r="J16" t="str">
-        <v>+91 9800000610</v>
+        <v>+91 9800000413</v>
       </c>
       <c r="K16">
         <v>5500000</v>
@@ -1070,39 +1070,39 @@
         <v>5500000</v>
       </c>
       <c r="M16" t="str">
-        <v>Flat A-610: Previous owner Jitender Kumar transferred to Sudheer Rai</v>
+        <v>Flat A-413: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹17,16,000) expired/renewed to Post-Possession Rate (@ ₹16,000/mo)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>701</v>
+        <v>501</v>
       </c>
       <c r="B17" t="str">
         <v>Tower A</v>
       </c>
       <c r="C17" t="str">
-        <v>Vandana Singh and Vinay Kumar Singh</v>
+        <v>Santokh Singh</v>
       </c>
       <c r="D17" t="str">
-        <v>+91 9800000701</v>
+        <v>+91 9800000501</v>
       </c>
       <c r="E17" t="str">
-        <v>16/10/2014</v>
+        <v>21/05/2014</v>
       </c>
       <c r="F17" t="str">
-        <v>15/12/2025</v>
+        <v>05/12/2025</v>
       </c>
       <c r="G17" t="str">
         <v>resale</v>
       </c>
       <c r="H17">
-        <v>1710000</v>
+        <v>1600000</v>
       </c>
       <c r="I17" t="str">
-        <v>Vimal Tripathi &amp; Namita Tripathi</v>
+        <v>Sunita Gupta</v>
       </c>
       <c r="J17" t="str">
-        <v>+91 9800000701</v>
+        <v>+91 9800000501</v>
       </c>
       <c r="K17">
         <v>5500000</v>
@@ -1111,39 +1111,39 @@
         <v>5500000</v>
       </c>
       <c r="M17" t="str">
-        <v>Flat A-701: Previous owner Vandana Singh and Vinay Kumar Singh transferred to Vimal Tripathi &amp; Namita Tripathi</v>
+        <v>Flat A-501: Prior owner Santokh Singh resold to Sunita Gupta</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>703</v>
+        <v>502</v>
       </c>
       <c r="B18" t="str">
         <v>Tower A</v>
       </c>
       <c r="C18" t="str">
-        <v>Rashmi Rekha Sahu</v>
+        <v>Amit Agarwal</v>
       </c>
       <c r="D18" t="str">
-        <v>+91 9800000703</v>
+        <v>+91 9800000502</v>
       </c>
       <c r="E18" t="str">
-        <v>08/01/2025</v>
+        <v>09/10/2014</v>
       </c>
       <c r="F18" t="str">
-        <v>14/06/2014</v>
+        <v>23/04/2025</v>
       </c>
       <c r="G18" t="str">
         <v>resale</v>
       </c>
       <c r="H18">
-        <v>1116000</v>
+        <v>1710000</v>
       </c>
       <c r="I18" t="str">
-        <v>Nirmala Devi</v>
+        <v>Jitender</v>
       </c>
       <c r="J18" t="str">
-        <v>+91 9800000703</v>
+        <v>+91 9800000502</v>
       </c>
       <c r="K18">
         <v>5500000</v>
@@ -1152,39 +1152,39 @@
         <v>5500000</v>
       </c>
       <c r="M18" t="str">
-        <v>Flat A-703: Previous owner Rashmi Rekha Sahu transferred to Nirmala Devi</v>
+        <v>Flat A-502: Prior owner Amit Agarwal resold to Jitender</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>706</v>
+        <v>503</v>
       </c>
       <c r="B19" t="str">
         <v>Tower A</v>
       </c>
       <c r="C19" t="str">
-        <v>Sukeshni Julka</v>
+        <v>Shefali Rani Mukherji</v>
       </c>
       <c r="D19" t="str">
-        <v>+91 9800000706</v>
+        <v>+91 9800000503</v>
       </c>
       <c r="E19" t="str">
-        <v>17/04/2015</v>
+        <v>13/03/2014</v>
       </c>
       <c r="F19" t="str">
-        <v>12/10/2025</v>
+        <v>21/01/2026</v>
       </c>
       <c r="G19" t="str">
         <v>resale</v>
       </c>
       <c r="H19">
-        <v>2000000</v>
+        <v>1600000</v>
       </c>
       <c r="I19" t="str">
-        <v>Brij Gopal Shah</v>
+        <v>Manju Goyal</v>
       </c>
       <c r="J19" t="str">
-        <v>+91 9800000706</v>
+        <v>+91 9800000503</v>
       </c>
       <c r="K19">
         <v>5500000</v>
@@ -1193,39 +1193,39 @@
         <v>5500000</v>
       </c>
       <c r="M19" t="str">
-        <v>Flat A-706: Previous owner Sukeshni Julka transferred to Brij Gopal Shah</v>
+        <v>Flat A-503: Prior owner Shefali Rani Mukherji resold to Manju Goyal</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>708</v>
+        <v>507</v>
       </c>
       <c r="B20" t="str">
         <v>Tower A</v>
       </c>
       <c r="C20" t="str">
-        <v>Varsha Gupta</v>
+        <v>Veena Sahani</v>
       </c>
       <c r="D20" t="str">
-        <v>+91 9800000708</v>
+        <v>+91 9800000507</v>
       </c>
       <c r="E20" t="str">
-        <v>13/03/2014</v>
+        <v>05/07/2014</v>
       </c>
       <c r="F20" t="str">
-        <v>04/04/2026</v>
+        <v>10/07/2024</v>
       </c>
       <c r="G20" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H20">
         <v>1600000</v>
       </c>
       <c r="I20" t="str">
-        <v>Monika Sharma</v>
+        <v>Veena Sahani</v>
       </c>
       <c r="J20" t="str">
-        <v>+91 9800000708</v>
+        <v>+91 9800000507</v>
       </c>
       <c r="K20">
         <v>5500000</v>
@@ -1234,39 +1234,39 @@
         <v>5500000</v>
       </c>
       <c r="M20" t="str">
-        <v>Flat A-708: Previous owner Varsha Gupta transferred to Monika Sharma</v>
+        <v>Flat A-507: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹16,00,000) expired/renewed to Post-Possession Rate (@ ₹16,000/mo)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>714</v>
+        <v>508</v>
       </c>
       <c r="B21" t="str">
         <v>Tower A</v>
       </c>
       <c r="C21" t="str">
-        <v>Kushum Shrivastva</v>
+        <v>Sanjay Madan and Sandhya Madan</v>
       </c>
       <c r="D21" t="str">
-        <v>+91 9800000714</v>
+        <v>+91 9800000508</v>
       </c>
       <c r="E21" t="str">
-        <v>24/06/2014</v>
+        <v>29/04/2014</v>
       </c>
       <c r="F21" t="str">
-        <v>15/12/2025</v>
+        <v>09/04/2025</v>
       </c>
       <c r="G21" t="str">
         <v>resale</v>
       </c>
       <c r="H21">
-        <v>1718000</v>
+        <v>1600000</v>
       </c>
       <c r="I21" t="str">
-        <v>Manish Sharma</v>
+        <v>Vishnu Kumar Agarwal</v>
       </c>
       <c r="J21" t="str">
-        <v>+91 9800000714</v>
+        <v>+91 9800000508</v>
       </c>
       <c r="K21">
         <v>5500000</v>
@@ -1275,39 +1275,39 @@
         <v>5500000</v>
       </c>
       <c r="M21" t="str">
-        <v>Flat A-714: Previous owner Kushum Shrivastva transferred to Manish Sharma</v>
+        <v>Flat A-508: Prior owner Sanjay Madan and Sandhya Madan resold to Vishnu Kumar Agarwal</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>801</v>
+        <v>512</v>
       </c>
       <c r="B22" t="str">
         <v>Tower A</v>
       </c>
       <c r="C22" t="str">
-        <v>Bhawna Babbar</v>
+        <v>Salman Shakeel</v>
       </c>
       <c r="D22" t="str">
-        <v>+91 9800000801</v>
+        <v>+91 9800000512</v>
       </c>
       <c r="E22" t="str">
-        <v>10/07/2014</v>
+        <v>30/03/2015</v>
       </c>
       <c r="F22" t="str">
-        <v>25/08/2025</v>
+        <v>10/04/2025</v>
       </c>
       <c r="G22" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H22">
-        <v>1600000</v>
+        <v>2200000</v>
       </c>
       <c r="I22" t="str">
-        <v>Mohini Choudhary</v>
+        <v>Salman Shakeel</v>
       </c>
       <c r="J22" t="str">
-        <v>+91 9800000801</v>
+        <v>+91 9800000512</v>
       </c>
       <c r="K22">
         <v>5500000</v>
@@ -1316,39 +1316,39 @@
         <v>5500000</v>
       </c>
       <c r="M22" t="str">
-        <v>Flat A-801: Previous owner Bhawna Babbar transferred to Mohini Choudhary</v>
+        <v>Flat A-512: Pre-Possession Contract (100mo @ ₹22000/mo, Total: ₹22,00,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>803</v>
+        <v>603</v>
       </c>
       <c r="B23" t="str">
         <v>Tower A</v>
       </c>
       <c r="C23" t="str">
-        <v>Satyajeet Sharma</v>
+        <v>Akshay Khullar</v>
       </c>
       <c r="D23" t="str">
-        <v>+91 9800000803</v>
+        <v>+91 9800000603</v>
       </c>
       <c r="E23" t="str">
-        <v>10/11/2025</v>
+        <v>13/03/2014</v>
       </c>
       <c r="F23" t="str">
-        <v>14/10/2014</v>
+        <v>09/04/2025</v>
       </c>
       <c r="G23" t="str">
         <v>resale</v>
       </c>
       <c r="H23">
-        <v>1860000</v>
+        <v>1600000</v>
       </c>
       <c r="I23" t="str">
-        <v>Manish Ganglani</v>
+        <v>Pooja Chand Dwivedi</v>
       </c>
       <c r="J23" t="str">
-        <v>+91 9800000803</v>
+        <v>+91 9800000603</v>
       </c>
       <c r="K23">
         <v>5500000</v>
@@ -1357,24 +1357,24 @@
         <v>5500000</v>
       </c>
       <c r="M23" t="str">
-        <v>Flat A-803: Previous owner Satyajeet Sharma transferred to Manish Ganglani</v>
+        <v>Flat A-603: Prior owner Akshay Khullar resold to Pooja Chand Dwivedi</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>805</v>
+        <v>606</v>
       </c>
       <c r="B24" t="str">
         <v>Tower A</v>
       </c>
       <c r="C24" t="str">
-        <v>Rita Chib</v>
+        <v>Rajeev Varshney</v>
       </c>
       <c r="D24" t="str">
-        <v>+91 9800000805</v>
+        <v>+91 9800000606</v>
       </c>
       <c r="E24" t="str">
-        <v>25/05/2015</v>
+        <v>10/10/2014</v>
       </c>
       <c r="F24" t="str">
         <v>21/11/2025</v>
@@ -1383,13 +1383,13 @@
         <v>resale</v>
       </c>
       <c r="H24">
-        <v>2200000</v>
+        <v>1591800</v>
       </c>
       <c r="I24" t="str">
-        <v>Punam Kumari Thakur</v>
+        <v>Praveen Tripathi</v>
       </c>
       <c r="J24" t="str">
-        <v>+91 9800000805</v>
+        <v>+91 9800000606</v>
       </c>
       <c r="K24">
         <v>5500000</v>
@@ -1398,39 +1398,39 @@
         <v>5500000</v>
       </c>
       <c r="M24" t="str">
-        <v>Flat A-805: Previous owner Rita Chib transferred to Punam Kumari Thakur</v>
+        <v>Flat A-606: Prior owner Rajeev Varshney resold to Praveen Tripathi</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>907</v>
+        <v>610</v>
       </c>
       <c r="B25" t="str">
         <v>Tower A</v>
       </c>
       <c r="C25" t="str">
-        <v>Ravi Shankar Venkatrama</v>
+        <v>Jitender Kumar</v>
       </c>
       <c r="D25" t="str">
-        <v>+91 9800000907</v>
+        <v>+91 9800000610</v>
       </c>
       <c r="E25" t="str">
-        <v>29/06/2014</v>
+        <v>21/10/2014</v>
       </c>
       <c r="F25" t="str">
-        <v>16/06/2025</v>
+        <v>13/03/2026</v>
       </c>
       <c r="G25" t="str">
         <v>resale</v>
       </c>
       <c r="H25">
-        <v>1722000</v>
+        <v>1875000</v>
       </c>
       <c r="I25" t="str">
-        <v>Sikha Srivastav</v>
+        <v>Sudheer Rai</v>
       </c>
       <c r="J25" t="str">
-        <v>+91 9800000907</v>
+        <v>+91 9800000610</v>
       </c>
       <c r="K25">
         <v>5500000</v>
@@ -1439,39 +1439,39 @@
         <v>5500000</v>
       </c>
       <c r="M25" t="str">
-        <v>Flat A-907: Previous owner Ravi Shankar Venkatrama transferred to Sikha Srivastav</v>
+        <v>Flat A-610: Prior owner Jitender Kumar resold to Sudheer Rai</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>909</v>
+        <v>612</v>
       </c>
       <c r="B26" t="str">
         <v>Tower A</v>
       </c>
       <c r="C26" t="str">
-        <v>Saurabh Jain</v>
+        <v>Uma Shankar Prasad Singh</v>
       </c>
       <c r="D26" t="str">
-        <v>+91 9800000909</v>
+        <v>+91 9800000612</v>
       </c>
       <c r="E26" t="str">
-        <v>04/12/2015</v>
+        <v>15/06/2015</v>
       </c>
       <c r="F26" t="str">
-        <v>01/01/2025</v>
+        <v>10/06/2025</v>
       </c>
       <c r="G26" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H26">
-        <v>2200000</v>
+        <v>2150000</v>
       </c>
       <c r="I26" t="str">
-        <v>Ashwar Gupta</v>
+        <v>Uma Shankar Prasad Singh</v>
       </c>
       <c r="J26" t="str">
-        <v>+91 9800000909</v>
+        <v>+91 9800000612</v>
       </c>
       <c r="K26">
         <v>5500000</v>
@@ -1480,39 +1480,39 @@
         <v>5500000</v>
       </c>
       <c r="M26" t="str">
-        <v>Flat A-909: Previous owner Saurabh Jain transferred to Ashwar Gupta</v>
+        <v>Flat A-612: Pre-Possession Contract (100mo @ ₹21500/mo, Total: ₹21,50,000) expired/renewed to Post-Possession Rate (@ ₹11,000/mo)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>1003</v>
+        <v>613</v>
       </c>
       <c r="B27" t="str">
         <v>Tower A</v>
       </c>
       <c r="C27" t="str">
-        <v>Raj Minocha</v>
+        <v>Sita Mathur</v>
       </c>
       <c r="D27" t="str">
-        <v>+91 9800001003</v>
+        <v>+91 9800000613</v>
       </c>
       <c r="E27" t="str">
-        <v>08/11/2013</v>
+        <v>31/07/2014</v>
       </c>
       <c r="F27" t="str">
-        <v>02/02/2026</v>
+        <v>10/07/2024</v>
       </c>
       <c r="G27" t="str">
-        <v>resale</v>
+        <v>pre_possession_contract</v>
       </c>
       <c r="H27">
-        <v>1600000</v>
+        <v>1716000</v>
       </c>
       <c r="I27" t="str">
-        <v>Rimpi Rani</v>
+        <v>Sita Mathur</v>
       </c>
       <c r="J27" t="str">
-        <v>+91 9800001003</v>
+        <v>+91 9800000613</v>
       </c>
       <c r="K27">
         <v>5500000</v>
@@ -1521,39 +1521,39 @@
         <v>5500000</v>
       </c>
       <c r="M27" t="str">
-        <v>Flat A-1003: Previous owner Raj Minocha transferred to Rimpi Rani</v>
+        <v>Flat A-613: Pre-Possession Contract (100mo @ ₹16000/mo, Total: ₹17,16,000) expired/renewed to Post-Possession Rate (@ ₹10,000/mo)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>1006</v>
+        <v>701</v>
       </c>
       <c r="B28" t="str">
         <v>Tower A</v>
       </c>
       <c r="C28" t="str">
-        <v>Sharda Tara and Vipin Tara</v>
+        <v>Vandana Singh and Vinay Kumar Singh</v>
       </c>
       <c r="D28" t="str">
-        <v>+91 9800001006</v>
+        <v>+91 9800000701</v>
       </c>
       <c r="E28" t="str">
-        <v>21/03/2015</v>
+        <v>16/10/2014</v>
       </c>
       <c r="F28" t="str">
-        <v>10/11/2025</v>
+        <v>15/12/2025</v>
       </c>
       <c r="G28" t="str">
         <v>resale</v>
       </c>
       <c r="H28">
-        <v>2200000</v>
+        <v>1710000</v>
       </c>
       <c r="I28" t="str">
-        <v>Anju Sharma</v>
+        <v>Vimal Tripathi &amp; Namita Tripathi</v>
       </c>
       <c r="J28" t="str">
-        <v>+91 9800001006</v>
+        <v>+91 9800000701</v>
       </c>
       <c r="K28">
         <v>5500000</v>
@@ -1562,39 +1562,39 @@
         <v>5500000</v>
       </c>
       <c r="M28" t="str">
-        <v>Flat A-1006: Previous owner Sharda Tara and Vipin Tara transferred to Anju Sharma</v>
+        <v>Flat A-701: Prior owner Vandana Singh and Vinay Kumar Singh resold to Vimal Tripathi &amp; Namita Tripathi</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>1008</v>
+        <v>703</v>
       </c>
       <c r="B29" t="str">
         <v>Tower A</v>
       </c>
       <c r="C29" t="str">
-        <v>Shivendra Singh</v>
+        <v>Rashmi Rekha Sahu</v>
       </c>
       <c r="D29" t="str">
-        <v>+91 9800001008</v>
+        <v>+91 9800000703</v>
       </c>
       <c r="E29" t="str">
-        <v>12/10/2015</v>
+        <v>08/01/2025</v>
       </c>
       <c r="F29" t="str">
-        <v>22/12/2025</v>
+        <v>14/06/2014</v>
       </c>
       <c r="G29" t="str">
         <v>resale</v>
       </c>
       <c r="H29">
-        <v>2200000</v>
+        <v>1116000</v>
       </c>
       <c r="I29" t="str">
-        <v>Sangeeta Chaturvedi</v>
+        <v>Nirmala Devi</v>
       </c>
       <c r="J29" t="str">
-        <v>+91 9800001008</v>
+        <v>+91 9800000703</v>
       </c>
       <c r="K29">
         <v>5500000</v>
@@ -1603,53 +1603,586 @@
         <v>5500000</v>
       </c>
       <c r="M29" t="str">
-        <v>Flat A-1008: Previous owner Shivendra Singh transferred to Sangeeta Chaturvedi</v>
+        <v>Flat A-703: Prior owner Rashmi Rekha Sahu resold to Nirmala Devi</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
+        <v>706</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Sukeshni Julka</v>
+      </c>
+      <c r="D30" t="str">
+        <v>+91 9800000706</v>
+      </c>
+      <c r="E30" t="str">
+        <v>17/04/2015</v>
+      </c>
+      <c r="F30" t="str">
+        <v>12/10/2025</v>
+      </c>
+      <c r="G30" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H30">
+        <v>2000000</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Brij Gopal Shah</v>
+      </c>
+      <c r="J30" t="str">
+        <v>+91 9800000706</v>
+      </c>
+      <c r="K30">
+        <v>5500000</v>
+      </c>
+      <c r="L30">
+        <v>5500000</v>
+      </c>
+      <c r="M30" t="str">
+        <v>Flat A-706: Prior owner Sukeshni Julka resold to Brij Gopal Shah</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>708</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Varsha Gupta</v>
+      </c>
+      <c r="D31" t="str">
+        <v>+91 9800000708</v>
+      </c>
+      <c r="E31" t="str">
+        <v>13/03/2014</v>
+      </c>
+      <c r="F31" t="str">
+        <v>04/04/2026</v>
+      </c>
+      <c r="G31" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H31">
+        <v>1600000</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Monika Sharma</v>
+      </c>
+      <c r="J31" t="str">
+        <v>+91 9800000708</v>
+      </c>
+      <c r="K31">
+        <v>5500000</v>
+      </c>
+      <c r="L31">
+        <v>5500000</v>
+      </c>
+      <c r="M31" t="str">
+        <v>Flat A-708: Prior owner Varsha Gupta resold to Monika Sharma</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>714</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Kushum Shrivastva</v>
+      </c>
+      <c r="D32" t="str">
+        <v>+91 9800000714</v>
+      </c>
+      <c r="E32" t="str">
+        <v>24/06/2014</v>
+      </c>
+      <c r="F32" t="str">
+        <v>15/12/2025</v>
+      </c>
+      <c r="G32" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H32">
+        <v>1718000</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Manish Sharma</v>
+      </c>
+      <c r="J32" t="str">
+        <v>+91 9800000714</v>
+      </c>
+      <c r="K32">
+        <v>5500000</v>
+      </c>
+      <c r="L32">
+        <v>5500000</v>
+      </c>
+      <c r="M32" t="str">
+        <v>Flat A-714: Prior owner Kushum Shrivastva resold to Manish Sharma</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>801</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Bhawna Babbar</v>
+      </c>
+      <c r="D33" t="str">
+        <v>+91 9800000801</v>
+      </c>
+      <c r="E33" t="str">
+        <v>10/07/2014</v>
+      </c>
+      <c r="F33" t="str">
+        <v>25/08/2025</v>
+      </c>
+      <c r="G33" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H33">
+        <v>1600000</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Mohini Choudhary</v>
+      </c>
+      <c r="J33" t="str">
+        <v>+91 9800000801</v>
+      </c>
+      <c r="K33">
+        <v>5500000</v>
+      </c>
+      <c r="L33">
+        <v>5500000</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Flat A-801: Prior owner Bhawna Babbar resold to Mohini Choudhary</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>803</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Satyajeet Sharma</v>
+      </c>
+      <c r="D34" t="str">
+        <v>+91 9800000803</v>
+      </c>
+      <c r="E34" t="str">
+        <v>10/11/2025</v>
+      </c>
+      <c r="F34" t="str">
+        <v>14/10/2014</v>
+      </c>
+      <c r="G34" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H34">
+        <v>1860000</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Manish Ganglani</v>
+      </c>
+      <c r="J34" t="str">
+        <v>+91 9800000803</v>
+      </c>
+      <c r="K34">
+        <v>5500000</v>
+      </c>
+      <c r="L34">
+        <v>5500000</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Flat A-803: Prior owner Satyajeet Sharma resold to Manish Ganglani</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>805</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Rita Chib</v>
+      </c>
+      <c r="D35" t="str">
+        <v>+91 9800000805</v>
+      </c>
+      <c r="E35" t="str">
+        <v>25/05/2015</v>
+      </c>
+      <c r="F35" t="str">
+        <v>21/11/2025</v>
+      </c>
+      <c r="G35" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H35">
+        <v>2200000</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Punam Kumari Thakur</v>
+      </c>
+      <c r="J35" t="str">
+        <v>+91 9800000805</v>
+      </c>
+      <c r="K35">
+        <v>5500000</v>
+      </c>
+      <c r="L35">
+        <v>5500000</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Flat A-805: Prior owner Rita Chib resold to Punam Kumari Thakur</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>806</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Ruchi Kulshreshtha</v>
+      </c>
+      <c r="D36" t="str">
+        <v>+91 9800000806</v>
+      </c>
+      <c r="E36" t="str">
+        <v>15/04/2015</v>
+      </c>
+      <c r="F36" t="str">
+        <v>10/04/2025</v>
+      </c>
+      <c r="G36" t="str">
+        <v>pre_possession_contract</v>
+      </c>
+      <c r="H36">
+        <v>2200000</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Ruchi Kulshreshtha</v>
+      </c>
+      <c r="J36" t="str">
+        <v>+91 9800000806</v>
+      </c>
+      <c r="K36">
+        <v>5500000</v>
+      </c>
+      <c r="L36">
+        <v>5500000</v>
+      </c>
+      <c r="M36" t="str">
+        <v>Flat A-806: Pre-Possession Contract (100mo @ ₹22000/mo, Total: ₹22,00,000) expired/renewed to Post-Possession Rate (@ ₹10,000/mo)</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>906</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Satyajeet Sharma</v>
+      </c>
+      <c r="D37" t="str">
+        <v>+91 9800000906</v>
+      </c>
+      <c r="E37" t="str">
+        <v>17/09/2015</v>
+      </c>
+      <c r="F37" t="str">
+        <v>10/11/2023</v>
+      </c>
+      <c r="G37" t="str">
+        <v>pre_possession_contract</v>
+      </c>
+      <c r="H37">
+        <v>1767200</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Satyajeet Sharma</v>
+      </c>
+      <c r="J37" t="str">
+        <v>+91 9800000906</v>
+      </c>
+      <c r="K37">
+        <v>5500000</v>
+      </c>
+      <c r="L37">
+        <v>5500000</v>
+      </c>
+      <c r="M37" t="str">
+        <v>Flat A-906: Pre-Possession Contract (100mo @ ₹20972/mo, Total: ₹17,67,200) expired/renewed to Post-Possession Rate (@ ₹20,972/mo)</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>907</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Ravi Shankar Venkatrama</v>
+      </c>
+      <c r="D38" t="str">
+        <v>+91 9800000907</v>
+      </c>
+      <c r="E38" t="str">
+        <v>29/06/2014</v>
+      </c>
+      <c r="F38" t="str">
+        <v>16/06/2025</v>
+      </c>
+      <c r="G38" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H38">
+        <v>1722000</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Sikha Srivastav</v>
+      </c>
+      <c r="J38" t="str">
+        <v>+91 9800000907</v>
+      </c>
+      <c r="K38">
+        <v>5500000</v>
+      </c>
+      <c r="L38">
+        <v>5500000</v>
+      </c>
+      <c r="M38" t="str">
+        <v>Flat A-907: Prior owner Ravi Shankar Venkatrama resold to Sikha Srivastav</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>909</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Saurabh Jain</v>
+      </c>
+      <c r="D39" t="str">
+        <v>+91 9800000909</v>
+      </c>
+      <c r="E39" t="str">
+        <v>04/12/2015</v>
+      </c>
+      <c r="F39" t="str">
+        <v>01/01/2025</v>
+      </c>
+      <c r="G39" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H39">
+        <v>2200000</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Ashwar Gupta</v>
+      </c>
+      <c r="J39" t="str">
+        <v>+91 9800000909</v>
+      </c>
+      <c r="K39">
+        <v>5500000</v>
+      </c>
+      <c r="L39">
+        <v>5500000</v>
+      </c>
+      <c r="M39" t="str">
+        <v>Flat A-909: Prior owner Saurabh Jain resold to Ashwar Gupta</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>1003</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Raj Minocha</v>
+      </c>
+      <c r="D40" t="str">
+        <v>+91 9800001003</v>
+      </c>
+      <c r="E40" t="str">
+        <v>08/11/2013</v>
+      </c>
+      <c r="F40" t="str">
+        <v>02/02/2026</v>
+      </c>
+      <c r="G40" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H40">
+        <v>1600000</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Rimpi Rani</v>
+      </c>
+      <c r="J40" t="str">
+        <v>+91 9800001003</v>
+      </c>
+      <c r="K40">
+        <v>5500000</v>
+      </c>
+      <c r="L40">
+        <v>5500000</v>
+      </c>
+      <c r="M40" t="str">
+        <v>Flat A-1003: Prior owner Raj Minocha resold to Rimpi Rani</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>1006</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Sharda Tara and Vipin Tara</v>
+      </c>
+      <c r="D41" t="str">
+        <v>+91 9800001006</v>
+      </c>
+      <c r="E41" t="str">
+        <v>21/03/2015</v>
+      </c>
+      <c r="F41" t="str">
+        <v>10/11/2025</v>
+      </c>
+      <c r="G41" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H41">
+        <v>2200000</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Anju Sharma</v>
+      </c>
+      <c r="J41" t="str">
+        <v>+91 9800001006</v>
+      </c>
+      <c r="K41">
+        <v>5500000</v>
+      </c>
+      <c r="L41">
+        <v>5500000</v>
+      </c>
+      <c r="M41" t="str">
+        <v>Flat A-1006: Prior owner Sharda Tara and Vipin Tara resold to Anju Sharma</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>1008</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Shivendra Singh</v>
+      </c>
+      <c r="D42" t="str">
+        <v>+91 9800001008</v>
+      </c>
+      <c r="E42" t="str">
+        <v>12/10/2015</v>
+      </c>
+      <c r="F42" t="str">
+        <v>22/12/2025</v>
+      </c>
+      <c r="G42" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H42">
+        <v>2200000</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Sangeeta Chaturvedi</v>
+      </c>
+      <c r="J42" t="str">
+        <v>+91 9800001008</v>
+      </c>
+      <c r="K42">
+        <v>5500000</v>
+      </c>
+      <c r="L42">
+        <v>5500000</v>
+      </c>
+      <c r="M42" t="str">
+        <v>Flat A-1008: Prior owner Shivendra Singh resold to Sangeeta Chaturvedi</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
         <v>1009</v>
       </c>
-      <c r="B30" t="str">
-        <v>Tower A</v>
-      </c>
-      <c r="C30" t="str">
+      <c r="B43" t="str">
+        <v>Tower A</v>
+      </c>
+      <c r="C43" t="str">
         <v>Shivendra Singh</v>
       </c>
-      <c r="D30" t="str">
+      <c r="D43" t="str">
         <v>+91 9800001009</v>
       </c>
-      <c r="E30" t="str">
+      <c r="E43" t="str">
         <v>12/10/2015</v>
       </c>
-      <c r="F30" t="str">
+      <c r="F43" t="str">
         <v>22/12/2025</v>
       </c>
-      <c r="G30" t="str">
-        <v>resale</v>
-      </c>
-      <c r="H30">
+      <c r="G43" t="str">
+        <v>resale</v>
+      </c>
+      <c r="H43">
         <v>2200000</v>
       </c>
-      <c r="I30" t="str">
+      <c r="I43" t="str">
         <v>Sangeeta Chaturvedi</v>
       </c>
-      <c r="J30" t="str">
+      <c r="J43" t="str">
         <v>+91 9800001009</v>
       </c>
-      <c r="K30">
-        <v>5500000</v>
-      </c>
-      <c r="L30">
-        <v>5500000</v>
-      </c>
-      <c r="M30" t="str">
-        <v>Flat A-1009: Previous owner Shivendra Singh transferred to Sangeeta Chaturvedi</v>
+      <c r="K43">
+        <v>5500000</v>
+      </c>
+      <c r="L43">
+        <v>5500000</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Flat A-1009: Prior owner Shivendra Singh resold to Sangeeta Chaturvedi</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add resell, buy_back, and possession_renewal statuses across backend schema, excel importer, and frontend filters/badges
</commit_message>
<xml_diff>
--- a/Tower_A_Ownership_History_Resale_v2.xlsx
+++ b/Tower_A_Ownership_History_Resale_v2.xlsx
@@ -560,7 +560,7 @@
         <v>10/08/2024</v>
       </c>
       <c r="G4" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H4">
         <v>1600000</v>
@@ -683,7 +683,7 @@
         <v>10/01/2026</v>
       </c>
       <c r="G7" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H7">
         <v>1738600</v>
@@ -724,7 +724,7 @@
         <v>10/05/2025</v>
       </c>
       <c r="G8" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H8">
         <v>1456000</v>
@@ -765,7 +765,7 @@
         <v>10/05/2025</v>
       </c>
       <c r="G9" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H9">
         <v>1732000</v>
@@ -847,7 +847,7 @@
         <v>10/05/2025</v>
       </c>
       <c r="G11" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H11">
         <v>2200000</v>
@@ -888,7 +888,7 @@
         <v>10/02/2024</v>
       </c>
       <c r="G12" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H12">
         <v>1600000</v>
@@ -1052,7 +1052,7 @@
         <v>10/07/2024</v>
       </c>
       <c r="G16" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H16">
         <v>1716000</v>
@@ -1216,7 +1216,7 @@
         <v>10/07/2024</v>
       </c>
       <c r="G20" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H20">
         <v>1600000</v>
@@ -1298,7 +1298,7 @@
         <v>10/04/2025</v>
       </c>
       <c r="G22" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H22">
         <v>2200000</v>
@@ -1462,7 +1462,7 @@
         <v>10/06/2025</v>
       </c>
       <c r="G26" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H26">
         <v>2150000</v>
@@ -1503,7 +1503,7 @@
         <v>10/07/2024</v>
       </c>
       <c r="G27" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H27">
         <v>1716000</v>
@@ -1872,7 +1872,7 @@
         <v>10/04/2025</v>
       </c>
       <c r="G36" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H36">
         <v>2200000</v>
@@ -1913,7 +1913,7 @@
         <v>10/11/2023</v>
       </c>
       <c r="G37" t="str">
-        <v>pre_possession_contract</v>
+        <v>possession_renewal</v>
       </c>
       <c r="H37">
         <v>1767200</v>

</xml_diff>